<commit_message>
Update test results to accurately reflect transaction statuses
Update the test matrix artifact (xlsx) to include corrected transaction IDs, folio numbers, and statuses for both bill payment and mobile top-up test cases.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: cabc721f-c66c-4670-ad9f-a3c7bf5dd0cd
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 8947657c-65c7-4e99-aeb4-ae79e20daaa1
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/86cae774-c82e-441c-9e1e-162b1f174041/cabc721f-c66c-4670-ad9f-a3c7bf5dd0cd/xBqarTU
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/src/billpay/scripts/Matriz_Pruebas_PagoYa_Taecel_v3_FINAL.xlsx
+++ b/artifacts/api-server/src/billpay/scripts/Matriz_Pruebas_PagoYa_Taecel_v3_FINAL.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz TU" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle Completo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de Pruebas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle Técnico" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,11 +52,20 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00B45309"/>
+      <color rgb="0092400E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +75,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000A1628"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -105,13 +119,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -120,7 +134,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -128,12 +142,23 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,29 +524,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TABLA DE RESULTADOS — PagoYa / Taecel  |  Cuenta: ID373554  |  Fecha ejecución: 2026-05-07  |  Endpoint: https://api-v1-fixedip.taecel.com/api/</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+          <t>TABLA DE RESULTADOS — PagoYa / Taecel  |  Cuenta ID373554  |  BP ejecutado: 2026-04-30  |  TU ejecutado: 2026-05-07  |  Endpoint: https://api-v1-fixedip.taecel.com/api/</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ID</t>
@@ -529,22 +555,22 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Portador</t>
+          <t>Servicio</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Código (SKU)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Teléfono Ref.</t>
+          <t>Referencia</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Monto</t>
+          <t>Monto (MXN)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -570,48 +596,53 @@
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Tipo</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>TU-01</t>
+          <t>BP-01</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>TELCEL</t>
+          <t>SKY</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>TEL010</t>
+          <t>SKY000</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>3221839799</t>
+          <t>871235412635</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>$10</t>
+          <t>$95</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>260500409352</t>
+          <t>260401841047</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>196283</t>
+          <t>114532</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -621,49 +652,50 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Tiempo Aire</t>
-        </is>
-      </c>
+          <t>Pago de Servicios</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>TU-02</t>
+          <t>BP-02</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>TELCEL</t>
+          <t>TELMEX</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>TEL050</t>
+          <t>TMX001</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>5555555502</t>
+          <t>6589745213</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>$50</t>
+          <t>$100</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>260500409967</t>
+          <t>260401841055</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>141625</t>
+          <t>856925</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -673,49 +705,50 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Tiempo Aire</t>
-        </is>
-      </c>
+          <t>Pago de Servicios</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>TU-03</t>
+          <t>BP-03</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>TELCEL</t>
+          <t>CFE</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>TEL100</t>
+          <t>CFE000</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>5555555503</t>
+          <t>125478965412365478965230126654</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>$100</t>
+          <t>$260</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>260500409979</t>
+          <t>260401841069</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>526567</t>
+          <t>733392</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -725,49 +758,50 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Tiempo Aire</t>
-        </is>
-      </c>
+          <t>Pago de Servicios</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>TU-04</t>
+          <t>BP-04</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>TELCEL</t>
+          <t>MEGACABLE</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>TEL150</t>
+          <t>MEG000</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>5555555504</t>
+          <t>9854123547</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>$150</t>
+          <t>$131</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>260500409990</t>
+          <t>260401841081</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>821964</t>
+          <t>548928</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -777,333 +811,609 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Tiempo Aire</t>
-        </is>
-      </c>
+          <t>Pago de Servicios</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr"/>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>TU-05</t>
+          <t>BP-05</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>DISH</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>DSH000</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>27458965324125</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>$103</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>260401841092</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>521535</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Pago de Servicios</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>TU-01</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
           <t>TELCEL</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>TEL200</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>5555555505</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>$200</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>260500410007</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>525341</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>TEL010</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>3221839799</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>$10</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>260500409352</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>196283</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Tiempo Aire</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>TU-06</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>MOVISTAR</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>MOV010</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>3221923297</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>$10</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>260500409398</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>330902</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>TU-02</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>TELCEL</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>TEL050</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>5555555502</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>$50</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>260500409967</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>141625</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Tiempo Aire</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>TU-07</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>MOVISTAR</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>MOV050</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>5555555507</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>$50</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>260500410018</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>997200</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>TU-03</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>TELCEL</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>TEL100</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>5555555503</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>260500409979</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>526567</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>Tiempo Aire</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>TU-08</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>MOVISTAR</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>MOV100</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>5555555508</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>$100</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>260500410032</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>983930</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>TU-04</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>TELCEL</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>TEL150</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>5555555504</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>$150</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>260500409990</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>821964</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>Tiempo Aire</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>TU-09</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>MOVISTAR</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>MOV120</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>5555555509</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>$120</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>260500410039</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>491604</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Exitosa</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>Tiempo Aire</t>
-        </is>
-      </c>
+      <c r="K11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
+          <t>TU-05</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>TELCEL</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>TEL200</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>5555555505</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>$200</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>260500410007</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>525341</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Tiempo Aire</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>TU-06</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>MOVISTAR</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>MOV010</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>3221923297</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>$10</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>260500409398</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>330902</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>Tiempo Aire</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>TU-07</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>MOVISTAR</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>MOV050</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>5555555507</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>$50</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>260500410018</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>997200</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>Tiempo Aire</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>TU-08</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>MOVISTAR</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>MOV100</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>5555555508</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>260500410032</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>983930</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>Tiempo Aire</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>TU-09</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>MOVISTAR</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>MOV120</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>5555555509</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>$120</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>260500410039</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>491604</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Exitosa</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>Tiempo Aire</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
           <t>TU-10</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>MOVISTAR</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>MOV150</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>5555555200</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>$150</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="I17" s="11" t="inlineStr">
         <is>
           <t>Error 3129 (ESPERADO)</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="J17" s="9" t="inlineStr">
         <is>
           <t>Tiempo Aire</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Exitosa: 9  /  Error esperado (ESPERADO): 1  /  Total pruebas: 10  →  CERTIFICACIÓN COMPLETADA ✓</t>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>Tabla de transacciones llena — resultado esperado y certificado</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Exitosa: 14   |   Error esperado (ESPERADO): 1   |   Total pruebas: 15   |   Passed exitosa: 14   |   Expected errors: 1   |   Failures: 0   |   Timeouts: 0   |   Total: 15/15   →   CERTIFICACIÓN COMPLETADA ✓</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A18:K18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1115,222 +1425,302 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Campo</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>MATRIZ DE PRUEBAS — DETALLE TÉCNICO</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ejecutado por</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>PagoYa — agente automatizado vía Node.js fetch</t>
-        </is>
-      </c>
+      <c r="A2" s="13" t="inlineStr"/>
+      <c r="B2" s="14" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Fecha ejecución</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Empresa</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>PagoYa</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Cuenta Taecel</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>ID373554</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>https://api-v1-fixedip.taecel.com/api/</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Cuenta Taecel</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ID373554</t>
-        </is>
-      </c>
-    </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Método de ejecución</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Node.js 24 / fetch — pnpm exec tsx</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr"/>
+      <c r="B7" s="14" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>── PAGO DE SERVICIOS (BP) — 2026-04-30 ──</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>BP-01</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>SKY | SKY000 | Ref: 871235412635 | $95 | TransID: 260401841047 | Folio: 114532 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>BP-02</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>TELMEX | TMX001 | Ref: 6589745213 | $100 | TransID: 260401841055 | Folio: 856925 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>BP-03</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>CFE | CFE000 | Ref: 125478965412365478965230126654 | $260 | TransID: 260401841069 | Folio: 733392 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>BP-04</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>MEGACABLE | MEG000 | Ref: 9854123547 | $131 | TransID: 260401841081 | Folio: 548928 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>BP-05</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>DISH | DSH000 | Ref: 27458965324125 | $103 | TransID: 260401841092 | Folio: 521535 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr"/>
+      <c r="B14" s="14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>── TIEMPO AIRE (TU) — 2026-05-07 ──</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>TU-01</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>TELCEL TEL010 | Ref: 3221839799 | $10 | TransID: 260500409352 | Folio: 196283 | ✅ Exitosa</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>TELCEL | TEL010 | Ref: 3221839799 | $10 | TransID: 260500409352 | Folio: 196283 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>TU-02</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>TELCEL TEL050 | Ref: 5555555502 | $50 | TransID: 260500409967 | Folio: 141625 | ✅ Exitosa</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>TELCEL | TEL050 | Ref: 5555555502 | $50 | TransID: 260500409967 | Folio: 141625 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>TU-03</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>TELCEL TEL100 | Ref: 5555555503 | $100 | TransID: 260500409979 | Folio: 526567 | ✅ Exitosa</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>TELCEL | TEL100 | Ref: 5555555503 | $100 | TransID: 260500409979 | Folio: 526567 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>TU-04</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>TELCEL TEL150 | Ref: 5555555504 | $150 | TransID: 260500409990 | Folio: 821964 | ✅ Exitosa</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>TELCEL | TEL150 | Ref: 5555555504 | $150 | TransID: 260500409990 | Folio: 821964 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>TU-05</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>TELCEL TEL200 | Ref: 5555555505 | $200 | TransID: 260500410007 | Folio: 525341 | ✅ Exitosa</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>TELCEL | TEL200 | Ref: 5555555505 | $200 | TransID: 260500410007 | Folio: 525341 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>TU-06</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>MOVISTAR MOV010 | Ref: 3221923297 | $10 | TransID: 260500409398 | Folio: 330902 | ✅ Exitosa</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>MOVISTAR | MOV010 | Ref: 3221923297 | $10 | TransID: 260500409398 | Folio: 330902 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>TU-07</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>MOVISTAR MOV050 | Ref: 5555555507 | $50 | TransID: 260500410018 | Folio: 997200 | ✅ Exitosa</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>MOVISTAR | MOV050 | Ref: 5555555507 | $50 | TransID: 260500410018 | Folio: 997200 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>TU-08</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>MOVISTAR MOV100 | Ref: 5555555508 | $100 | TransID: 260500410032 | Folio: 983930 | ✅ Exitosa</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>MOVISTAR | MOV100 | Ref: 5555555508 | $100 | TransID: 260500410032 | Folio: 983930 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>TU-09</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>MOVISTAR MOV120 | Ref: 5555555509 | $120 | TransID: 260500410039 | Folio: 491604 | ✅ Exitosa</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>MOVISTAR | MOV120 | Ref: 5555555509 | $120 | TransID: 260500410039 | Folio: 491604 | Exitosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>TU-10</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>MOVISTAR MOV150 | Ref: 5555555200 | $150 | TransID: — | Folio: — | ✅ Error 3129 (ESPERADO) — Tabla de transacciones llena</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>MOVISTAR | MOV150 | Ref: 5555555200 | $150 | TransID: — | Folio: — | Error 3129 (ESPERADO) — Tabla de transacciones llena</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr"/>
+      <c r="B26" s="14" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Nota TU-10</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Error 3129 es el comportamiento esperado y certificado. MOV150 devuelve 'Tabla de transacciones llena' por diseño de Taecel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>Error 3129 'Tabla de transacciones llena' es el resultado correcto y esperado para MOV150 según la matriz de certificación Taecel. No es un fallo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>Resultado final</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>10/10 pruebas superadas. Certificación Taecel completada.</t>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>15/15 pruebas superadas. Certificación Taecel completada.</t>
         </is>
       </c>
     </row>

</xml_diff>